<commit_message>
Updated citation language and removed SEENDTC from output variables.
</commit_message>
<xml_diff>
--- a/rules/CORE-000352/negative/01/data/unit-test-coreid-CG0207-negative.xlsx
+++ b/rules/CORE-000352/negative/01/data/unit-test-coreid-CG0207-negative.xlsx
@@ -480,7 +480,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
       <c r="B2" s="4" t="str">
@@ -507,10 +507,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>se.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Subject Elements</v>
       </c>
     </row>
@@ -523,7 +523,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -546,128 +546,88 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>se.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
+        <v>6</v>
+      </c>
+      <c r="E2" s="4" t="str">
+        <v>SESTDTC</v>
+      </c>
+      <c r="F2" s="4" t="str">
+        <v>2012-11-31</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="str">
+        <v>se.xpt</v>
+      </c>
+      <c r="C3" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D3" s="4">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="str">
-        <v>SEENDTC</v>
-      </c>
-      <c r="F2" s="2" t="str">
-        <v>2012-11-30</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="str">
+      <c r="E3" s="4" t="str">
+        <v>ETCD</v>
+      </c>
+      <c r="F3" s="4" t="str">
+        <v>SCREEN</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="str">
         <v>se.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C4" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="2">
-        <v>6</v>
-      </c>
-      <c r="E3" s="2" t="str">
+      <c r="D4" s="4">
+        <v>8</v>
+      </c>
+      <c r="E4" s="4" t="str">
         <v>SESTDTC</v>
       </c>
-      <c r="F3" s="2" t="str">
-        <v>2012-11-31</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2">
-        <v>1</v>
-      </c>
-      <c r="B4" s="2" t="str">
+      <c r="F4" s="4" t="str">
+        <v>2012-11-16</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="str">
         <v>se.xpt</v>
       </c>
-      <c r="C4" s="2" t="str">
+      <c r="C5" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D4" s="2">
-        <v>5</v>
-      </c>
-      <c r="E4" s="2" t="str">
+      <c r="D5" s="4">
+        <v>7</v>
+      </c>
+      <c r="E5" s="4" t="str">
         <v>ETCD</v>
       </c>
-      <c r="F4" s="2" t="str">
-        <v>SCREEN</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2">
-        <v>2</v>
-      </c>
-      <c r="B5" s="2" t="str">
-        <v>se.xpt</v>
-      </c>
-      <c r="C5" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D5" s="2">
-        <v>7</v>
-      </c>
-      <c r="E5" s="2" t="str">
-        <v>SEENDTC</v>
-      </c>
-      <c r="F5" s="2" t="str">
-        <v>2012-11-15</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>2</v>
-      </c>
-      <c r="B6" s="2" t="str">
-        <v>se.xpt</v>
-      </c>
-      <c r="C6" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D6" s="2">
-        <v>8</v>
-      </c>
-      <c r="E6" s="2" t="str">
-        <v>SESTDTC</v>
-      </c>
-      <c r="F6" s="2" t="str">
-        <v>2012-11-16</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>2</v>
-      </c>
-      <c r="B7" s="2" t="str">
-        <v>se.xpt</v>
-      </c>
-      <c r="C7" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D7" s="2">
-        <v>7</v>
-      </c>
-      <c r="E7" s="2" t="str">
-        <v>ETCD</v>
-      </c>
-      <c r="F7" s="2" t="str">
+      <c r="F5" s="4" t="str">
         <v>SCREEN</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -841,7 +801,7 @@
       <c r="H5" s="4" t="str">
         <v>2012-11-23</v>
       </c>
-      <c r="I5" s="8" t="str">
+      <c r="I5" s="4" t="str">
         <v>2012-11-30</v>
       </c>
       <c r="J5" s="4">
@@ -873,7 +833,7 @@
       <c r="G6" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="H6" s="7" t="str">
+      <c r="H6" s="8" t="str">
         <v>2012-11-31</v>
       </c>
       <c r="I6" s="4" t="str">
@@ -899,7 +859,7 @@
       <c r="D7" s="4">
         <v>1</v>
       </c>
-      <c r="E7" s="7" t="str">
+      <c r="E7" s="8" t="str">
         <v>SCREEN</v>
       </c>
       <c r="F7" s="4" t="str">
@@ -911,7 +871,7 @@
       <c r="H7" s="4" t="str">
         <v>2012-10-30</v>
       </c>
-      <c r="I7" s="7" t="str">
+      <c r="I7" s="4" t="str">
         <v>2012-11-15</v>
       </c>
       <c r="J7" s="4">
@@ -943,7 +903,7 @@
       <c r="G8" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="H8" s="7" t="str">
+      <c r="H8" s="8" t="str">
         <v>2012-11-16</v>
       </c>
       <c r="I8" s="4" t="str">

</xml_diff>